<commit_message>
Fix #NAME? errors in roadmap Excel from prose starting with =
Excel treated explanation text like "= In Field Sets ÷ ..." as formulas.
Prefix those cells with "Formula:" so they display as text.

Co-authored-by: echenry6f <echenry6f@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/GSF_Utilization_Algorithm_Roadmap.xlsx
+++ b/GSF_Utilization_Algorithm_Roadmap.xlsx
@@ -178,7 +178,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -307,11 +307,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -419,6 +463,8 @@
     <xf numFmtId="0" fontId="14" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -842,6 +888,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
@@ -849,6 +896,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
@@ -913,27 +961,46 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Total Jobs</t>
         </is>
       </c>
+      <c r="B12" s="49" t="n"/>
+      <c r="C12" s="50" t="n"/>
       <c r="E12" s="17" t="inlineStr">
         <is>
           <t>GSF Jobs  =  In Field Sets  =  People Saved</t>
         </is>
       </c>
+      <c r="F12" s="49" t="n"/>
+      <c r="G12" s="49" t="n"/>
+      <c r="H12" s="49" t="n"/>
+      <c r="I12" s="49" t="n"/>
+      <c r="J12" s="49" t="n"/>
+      <c r="K12" s="50" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="18">
-        <f> COUNT of filtered Roads rows</f>
-        <v/>
-      </c>
-      <c r="E13" s="19">
-        <f> COUNTIFS(GSF Job, "Yes")   // 1 set per GSF job-day, not per AFD device</f>
-        <v/>
-      </c>
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Formula: COUNT of filtered Roads rows</t>
+        </is>
+      </c>
+      <c r="B13" s="51" t="n"/>
+      <c r="C13" s="52" t="n"/>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>Formula: COUNTIFS(GSF Job, "Yes")   // 1 set per GSF job-day, not per AFD device</t>
+        </is>
+      </c>
+      <c r="F13" s="51" t="n"/>
+      <c r="G13" s="51" t="n"/>
+      <c r="H13" s="51" t="n"/>
+      <c r="I13" s="51" t="n"/>
+      <c r="J13" s="51" t="n"/>
+      <c r="K13" s="52" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
@@ -959,18 +1026,40 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Sets on Hand (Working Days)</t>
         </is>
       </c>
+      <c r="B17" s="49" t="n"/>
+      <c r="C17" s="49" t="n"/>
+      <c r="D17" s="49" t="n"/>
+      <c r="E17" s="49" t="n"/>
+      <c r="F17" s="49" t="n"/>
+      <c r="G17" s="49" t="n"/>
+      <c r="H17" s="49" t="n"/>
+      <c r="I17" s="49" t="n"/>
+      <c r="J17" s="49" t="n"/>
+      <c r="K17" s="50" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="19">
-        <f> S × W   = physical sets × weekday working days (Mon–Fri only)</f>
-        <v/>
-      </c>
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>Formula: S × W   = physical sets × weekday working days (Mon–Fri only)</t>
+        </is>
+      </c>
+      <c r="B18" s="51" t="n"/>
+      <c r="C18" s="51" t="n"/>
+      <c r="D18" s="51" t="n"/>
+      <c r="E18" s="51" t="n"/>
+      <c r="F18" s="51" t="n"/>
+      <c r="G18" s="51" t="n"/>
+      <c r="H18" s="51" t="n"/>
+      <c r="I18" s="51" t="n"/>
+      <c r="J18" s="51" t="n"/>
+      <c r="K18" s="52" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="20" t="inlineStr">
@@ -993,36 +1082,52 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
           <t>GSF Utilization %</t>
         </is>
       </c>
+      <c r="B23" s="49" t="n"/>
+      <c r="C23" s="50" t="n"/>
       <c r="E23" s="17" t="inlineStr">
         <is>
           <t>GSF infield set / total jobs %</t>
         </is>
       </c>
+      <c r="F23" s="49" t="n"/>
+      <c r="G23" s="50" t="n"/>
       <c r="I23" s="17" t="inlineStr">
         <is>
           <t>People Saved</t>
         </is>
       </c>
+      <c r="J23" s="49" t="n"/>
+      <c r="K23" s="50" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="21">
-        <f> In Field Sets ÷ Sets on Hand</f>
-        <v/>
-      </c>
-      <c r="E24" s="21">
-        <f> GSF Jobs ÷ Total Jobs</f>
-        <v/>
-      </c>
-      <c r="I24" s="21">
-        <f> GSF In Field Sets</f>
-        <v/>
-      </c>
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>Formula: In Field Sets ÷ Sets on Hand</t>
+        </is>
+      </c>
+      <c r="B24" s="49" t="n"/>
+      <c r="C24" s="50" t="n"/>
+      <c r="E24" s="21" t="inlineStr">
+        <is>
+          <t>Formula: GSF Jobs ÷ Total Jobs</t>
+        </is>
+      </c>
+      <c r="F24" s="49" t="n"/>
+      <c r="G24" s="50" t="n"/>
+      <c r="I24" s="21" t="inlineStr">
+        <is>
+          <t>Formula: GSF In Field Sets</t>
+        </is>
+      </c>
+      <c r="J24" s="49" t="n"/>
+      <c r="K24" s="50" t="n"/>
     </row>
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="22" t="inlineStr">
@@ -1031,19 +1136,26 @@
 Washington: 14÷(6×5)=47%</t>
         </is>
       </c>
+      <c r="B25" s="49" t="n"/>
+      <c r="C25" s="50" t="n"/>
       <c r="E25" s="22" t="inlineStr">
         <is>
           <t>LOCKED
 (job-day counts)</t>
         </is>
       </c>
+      <c r="F25" s="49" t="n"/>
+      <c r="G25" s="50" t="n"/>
       <c r="I25" s="22" t="inlineStr">
         <is>
           <t>LOCKED
 (same number)</t>
         </is>
       </c>
-    </row>
+      <c r="J25" s="49" t="n"/>
+      <c r="K25" s="50" t="n"/>
+    </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="23" t="inlineStr">
         <is>
@@ -1058,12 +1170,23 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="25" t="inlineStr">
         <is>
           <t>Flagging Crews ≈ SUM(Assignment Count) [excl. Internal Labour?] [/2?]</t>
         </is>
       </c>
+      <c r="B30" s="51" t="n"/>
+      <c r="C30" s="51" t="n"/>
+      <c r="D30" s="51" t="n"/>
+      <c r="E30" s="51" t="n"/>
+      <c r="F30" s="51" t="n"/>
+      <c r="G30" s="51" t="n"/>
+      <c r="H30" s="51" t="n"/>
+      <c r="I30" s="51" t="n"/>
+      <c r="J30" s="51" t="n"/>
+      <c r="K30" s="52" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="25" t="inlineStr">
@@ -1071,19 +1194,35 @@
           <t>Total Crews ≈ SUM(Assignment Count) [all jobs, same unit basis]</t>
         </is>
       </c>
-    </row>
+      <c r="B31" s="51" t="n"/>
+      <c r="C31" s="51" t="n"/>
+      <c r="D31" s="51" t="n"/>
+      <c r="E31" s="51" t="n"/>
+      <c r="F31" s="51" t="n"/>
+      <c r="G31" s="51" t="n"/>
+      <c r="H31" s="51" t="n"/>
+      <c r="I31" s="51" t="n"/>
+      <c r="J31" s="51" t="n"/>
+      <c r="K31" s="52" t="n"/>
+    </row>
+    <row r="32"/>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
           <t>Fulfillment % = In Field Sets ÷ Flagging Crews</t>
         </is>
       </c>
+      <c r="B33" s="49" t="n"/>
+      <c r="C33" s="50" t="n"/>
       <c r="E33" s="26" t="inlineStr">
         <is>
           <t>Integration % = Sets on Hand ÷ Flagging Crews</t>
         </is>
       </c>
-    </row>
+      <c r="F33" s="49" t="n"/>
+      <c r="G33" s="50" t="n"/>
+    </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
@@ -1113,9 +1252,9 @@
     <mergeCell ref="I23:K23"/>
     <mergeCell ref="I25:K25"/>
     <mergeCell ref="E12:K12"/>
-    <mergeCell ref="A7:C8"/>
     <mergeCell ref="E25:G25"/>
     <mergeCell ref="A35:L35"/>
+    <mergeCell ref="A7:C8"/>
     <mergeCell ref="I7:K8"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A10:L10"/>
@@ -1168,6 +1307,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -1288,6 +1428,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -1383,9 +1524,10 @@
           <t>In Field Sets</t>
         </is>
       </c>
-      <c r="C17" s="31">
-        <f> GSF Jobs (1 set / GSF job-day)</f>
-        <v/>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>Formula: GSF Jobs (1 set / GSF job-day)</t>
+        </is>
       </c>
       <c r="D17" s="30" t="inlineStr">
         <is>
@@ -1407,9 +1549,10 @@
           <t>People Saved</t>
         </is>
       </c>
-      <c r="C18" s="31">
-        <f> In Field Sets</f>
-        <v/>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>Formula: In Field Sets</t>
+        </is>
       </c>
       <c r="D18" s="32" t="inlineStr">
         <is>
@@ -1499,6 +1642,8 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -1734,6 +1879,8 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="24" t="inlineStr">
         <is>
@@ -1886,6 +2033,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
@@ -1985,9 +2133,10 @@
           <t>People Saved</t>
         </is>
       </c>
-      <c r="C7" s="31">
-        <f> GSF In Field Sets</f>
-        <v/>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>Formula: GSF In Field Sets</t>
+        </is>
       </c>
       <c r="D7" s="30" t="inlineStr">
         <is>
@@ -2188,6 +2337,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="39" t="inlineStr">
         <is>
@@ -2313,6 +2463,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="42" t="inlineStr">
         <is>
@@ -2326,6 +2477,8 @@
           <t>1. Filter Roads to Dispatching = office and Assignment Date in range</t>
         </is>
       </c>
+      <c r="B12" s="51" t="n"/>
+      <c r="C12" s="52" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="44" t="inlineStr">
@@ -2333,6 +2486,8 @@
           <t>2. Total Jobs = row count</t>
         </is>
       </c>
+      <c r="B13" s="51" t="n"/>
+      <c r="C13" s="52" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="43" t="inlineStr">
@@ -2340,6 +2495,8 @@
           <t>3. GSF Jobs = In Field Sets = People Saved = count(GSF Job="Yes")</t>
         </is>
       </c>
+      <c r="B14" s="51" t="n"/>
+      <c r="C14" s="52" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="44" t="inlineStr">
@@ -2347,6 +2504,8 @@
           <t>4. Obtain physical set count S from inventory</t>
         </is>
       </c>
+      <c r="B15" s="51" t="n"/>
+      <c r="C15" s="52" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="43" t="inlineStr">
@@ -2354,6 +2513,8 @@
           <t>5. W = number of Mon–Fri days in the inclusive period</t>
         </is>
       </c>
+      <c r="B16" s="51" t="n"/>
+      <c r="C16" s="52" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="44" t="inlineStr">
@@ -2361,6 +2522,8 @@
           <t>6. Sets on Hand = S × W</t>
         </is>
       </c>
+      <c r="B17" s="51" t="n"/>
+      <c r="C17" s="52" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="43" t="inlineStr">
@@ -2368,6 +2531,8 @@
           <t>7. Utilization % = In Field Sets ÷ Sets on Hand (round as GU does)</t>
         </is>
       </c>
+      <c r="B18" s="51" t="n"/>
+      <c r="C18" s="52" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="44" t="inlineStr">
@@ -2375,6 +2540,8 @@
           <t>8. Mix % = GSF Jobs ÷ Total Jobs</t>
         </is>
       </c>
+      <c r="B19" s="51" t="n"/>
+      <c r="C19" s="52" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="43" t="inlineStr">
@@ -2382,12 +2549,14 @@
           <t>9. Optionally apply crew rules when confirmed for that office</t>
         </is>
       </c>
+      <c r="B20" s="51" t="n"/>
+      <c r="C20" s="52" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A19:C19"/>
     <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A19:C19"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A17:C17"/>
@@ -2422,6 +2591,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="45" t="inlineStr">
         <is>
@@ -2430,6 +2600,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="46" t="inlineStr">
         <is>
@@ -2469,6 +2640,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -2490,6 +2662,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>

</xml_diff>